<commit_message>
Refactor Actions.txt and documentation for improved clarity on global variables and processing logic. Introduced row override functionality for selective processing and enhanced error handling in SAP transactions. Updated frida-core.mdc and frida-sap.mdc with detailed guidelines on variable definitions and loop control. Removed temporary Excel file.
</commit_message>
<xml_diff>
--- a/Inputs/ECOM_MASIVO 9 FEBRERO 2026.xlsx
+++ b/Inputs/ECOM_MASIVO 9 FEBRERO 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodrigo.gracia\Documents\Projects\ECOM\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91544922-8DD7-42FA-929D-1B5B4A901D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE47AC3B-1E3E-4891-93E6-45C97017F73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26868" yWindow="9108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="3" r:id="rId1"/>
@@ -159,7 +159,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="194">
   <si>
     <t>ContractType</t>
   </si>
@@ -1135,6 +1135,39 @@
   </si>
   <si>
     <t>Material</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-02-27_16-44-30</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Characteristics: SAP(E) [ZACM000]: Incoterms 2 DAP is invalid</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Header Details (Basic):</t>
+  </si>
+  <si>
+    <t>SAPBot_2026-02-27_16-55-27</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1363,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1437,6 +1470,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1841,54 +1875,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E6F2E9B-55C0-40F5-AE06-67C582FE2E7E}">
-  <dimension ref="A1:AU18"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AW18"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="15" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.7265625" customWidth="1"/>
+    <col min="15" max="15" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="7.7265625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="9" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.7109375" customWidth="1"/>
-    <col min="37" max="37" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="43.28515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.7265625" customWidth="1"/>
+    <col min="37" max="37" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="43.26953125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="42" max="43" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="37.7265625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="26.81640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="56.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="37.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" ht="37.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2030,8 +2065,14 @@
       <c r="AU1" s="6" t="s">
         <v>34</v>
       </c>
+      <c r="AV1" t="s">
+        <v>183</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>184</v>
+      </c>
     </row>
-    <row r="2" spans="1:47" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>35</v>
       </c>
@@ -2124,8 +2165,11 @@
       <c r="AP2" s="39"/>
       <c r="AQ2" s="40"/>
       <c r="AU2" s="40"/>
+      <c r="AV2" t="s">
+        <v>185</v>
+      </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>35</v>
       </c>
@@ -2208,6 +2252,9 @@
       <c r="AI3" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ3">
+        <v>1000</v>
+      </c>
       <c r="AK3" s="36">
         <v>-5000</v>
       </c>
@@ -2236,8 +2283,14 @@
       <c r="AU3" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>192</v>
+      </c>
     </row>
-    <row r="4" spans="1:47" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:49" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -2329,6 +2382,9 @@
       <c r="AI4" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ4">
+        <v>1000</v>
+      </c>
       <c r="AK4" s="38">
         <v>100000</v>
       </c>
@@ -2354,8 +2410,14 @@
       <c r="AU4" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV4" t="s">
+        <v>191</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -2438,6 +2500,9 @@
       <c r="AI5" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ5">
+        <v>1000</v>
+      </c>
       <c r="AK5" s="38">
         <v>100000</v>
       </c>
@@ -2463,8 +2528,14 @@
       <c r="AU5" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV5" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -2540,6 +2611,9 @@
       <c r="AI6" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ6">
+        <v>1000</v>
+      </c>
       <c r="AL6" t="s">
         <v>58</v>
       </c>
@@ -2565,8 +2639,14 @@
       <c r="AU6" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV6" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -2642,6 +2722,9 @@
       <c r="AI7" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ7">
+        <v>1000</v>
+      </c>
       <c r="AL7" t="s">
         <v>58</v>
       </c>
@@ -2667,8 +2750,14 @@
       <c r="AU7" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV7" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -2748,6 +2837,9 @@
       <c r="AI8" s="34">
         <v>75.510000000000005</v>
       </c>
+      <c r="AJ8">
+        <v>1000</v>
+      </c>
       <c r="AL8" t="s">
         <v>179</v>
       </c>
@@ -2770,8 +2862,14 @@
       <c r="AU8" s="40" t="s">
         <v>65</v>
       </c>
+      <c r="AV8" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.35">
       <c r="C9" s="16"/>
       <c r="D9" s="17"/>
       <c r="I9" s="18"/>
@@ -2807,7 +2905,7 @@
       <c r="AT9" s="17"/>
       <c r="AU9" s="17"/>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.35">
       <c r="C10" s="16"/>
       <c r="I10" s="18"/>
       <c r="J10" s="18"/>
@@ -2843,7 +2941,7 @@
       <c r="AT10" s="17"/>
       <c r="AU10" s="17"/>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.35">
       <c r="C11" s="16"/>
       <c r="I11" s="18"/>
       <c r="J11" s="18"/>
@@ -2878,7 +2976,7 @@
       <c r="AT11" s="17"/>
       <c r="AU11" s="17"/>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.35">
       <c r="C12" s="16"/>
       <c r="I12" s="18"/>
       <c r="J12" s="18"/>
@@ -2914,7 +3012,7 @@
       <c r="AT12" s="17"/>
       <c r="AU12" s="17"/>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.35">
       <c r="C13" s="16"/>
       <c r="I13" s="18"/>
       <c r="J13" s="18"/>
@@ -2949,19 +3047,19 @@
       <c r="AT13" s="17"/>
       <c r="AU13" s="17"/>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.35">
       <c r="A16" s="23"/>
       <c r="B16" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="24"/>
       <c r="B17" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="25"/>
       <c r="B18" s="1" t="s">
         <v>128</v>
@@ -2976,23 +3074,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="6.7109375" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
-    <col min="8" max="9" width="16.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="33.85546875" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="6.7265625" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="9" width="16.81640625" customWidth="1"/>
+    <col min="10" max="10" width="11.81640625" customWidth="1"/>
+    <col min="11" max="11" width="33.81640625" customWidth="1"/>
+    <col min="12" max="12" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="27" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3028,6 +3126,139 @@
       </c>
       <c r="L1" s="3" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" s="41">
+        <v>46080.698923611111</v>
+      </c>
+      <c r="D2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="41">
+        <v>46080.699062500003</v>
+      </c>
+      <c r="D3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="41">
+        <v>46080.699236111112</v>
+      </c>
+      <c r="D4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" s="41">
+        <v>46080.69940972222</v>
+      </c>
+      <c r="D5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="41">
+        <v>46080.699571759258</v>
+      </c>
+      <c r="D6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="41">
+        <v>46080.699733796297</v>
+      </c>
+      <c r="D7" t="s">
+        <v>187</v>
+      </c>
+      <c r="E7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="41">
+        <v>46080.699895833335</v>
+      </c>
+      <c r="D8" t="s">
+        <v>187</v>
+      </c>
+      <c r="E8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C9" s="41">
+        <v>46080.705497685187</v>
+      </c>
+      <c r="D9" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3039,44 +3270,44 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AU18"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" style="1" customWidth="1"/>
     <col min="2" max="2" width="19" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" customWidth="1"/>
-    <col min="9" max="10" width="16.85546875" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
-    <col min="12" max="12" width="19.85546875" customWidth="1"/>
-    <col min="13" max="13" width="33.85546875" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" customWidth="1"/>
-    <col min="15" max="15" width="20.28515625" customWidth="1"/>
-    <col min="16" max="16" width="12.28515625" customWidth="1"/>
-    <col min="17" max="17" width="14.85546875" customWidth="1"/>
-    <col min="18" max="19" width="15.5703125" customWidth="1"/>
-    <col min="20" max="27" width="18.7109375" customWidth="1"/>
-    <col min="28" max="28" width="17.5703125" customWidth="1"/>
-    <col min="29" max="29" width="12.28515625" customWidth="1"/>
-    <col min="30" max="30" width="21.140625" customWidth="1"/>
-    <col min="31" max="32" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" customWidth="1"/>
+    <col min="6" max="6" width="6.7265625" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" customWidth="1"/>
+    <col min="8" max="8" width="9.81640625" customWidth="1"/>
+    <col min="9" max="10" width="16.81640625" customWidth="1"/>
+    <col min="11" max="11" width="11.81640625" customWidth="1"/>
+    <col min="12" max="12" width="19.81640625" customWidth="1"/>
+    <col min="13" max="13" width="33.81640625" customWidth="1"/>
+    <col min="14" max="14" width="10.7265625" customWidth="1"/>
+    <col min="15" max="15" width="20.26953125" customWidth="1"/>
+    <col min="16" max="16" width="12.26953125" customWidth="1"/>
+    <col min="17" max="17" width="14.81640625" customWidth="1"/>
+    <col min="18" max="19" width="15.54296875" customWidth="1"/>
+    <col min="20" max="27" width="18.7265625" customWidth="1"/>
+    <col min="28" max="28" width="17.54296875" customWidth="1"/>
+    <col min="29" max="29" width="12.26953125" customWidth="1"/>
+    <col min="30" max="30" width="21.1796875" customWidth="1"/>
+    <col min="31" max="32" width="12.26953125" customWidth="1"/>
     <col min="33" max="33" width="14" customWidth="1"/>
-    <col min="34" max="36" width="10.7109375" customWidth="1"/>
-    <col min="37" max="37" width="18.42578125" customWidth="1"/>
-    <col min="38" max="38" width="32.42578125" customWidth="1"/>
-    <col min="39" max="39" width="23.140625" customWidth="1"/>
-    <col min="40" max="40" width="28.140625" customWidth="1"/>
-    <col min="41" max="41" width="15.5703125" customWidth="1"/>
-    <col min="42" max="44" width="28.5703125" customWidth="1"/>
-    <col min="45" max="45" width="22.85546875" customWidth="1"/>
-    <col min="46" max="46" width="20.140625" customWidth="1"/>
-    <col min="47" max="47" width="28.5703125" customWidth="1"/>
+    <col min="34" max="36" width="10.7265625" customWidth="1"/>
+    <col min="37" max="37" width="18.453125" customWidth="1"/>
+    <col min="38" max="38" width="32.453125" customWidth="1"/>
+    <col min="39" max="39" width="23.1796875" customWidth="1"/>
+    <col min="40" max="40" width="28.1796875" customWidth="1"/>
+    <col min="41" max="41" width="15.54296875" customWidth="1"/>
+    <col min="42" max="44" width="28.54296875" customWidth="1"/>
+    <col min="45" max="45" width="22.81640625" customWidth="1"/>
+    <col min="46" max="46" width="20.1796875" customWidth="1"/>
+    <col min="47" max="47" width="28.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="37.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:47" ht="37.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3219,7 +3450,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>35</v>
       </c>
@@ -3355,7 +3586,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:47" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:47" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>35</v>
       </c>
@@ -3488,7 +3719,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -3625,7 +3856,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -3762,7 +3993,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -3899,7 +4130,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -4036,7 +4267,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -4173,7 +4404,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
@@ -4310,7 +4541,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>35</v>
       </c>
@@ -4447,7 +4678,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>35</v>
       </c>
@@ -4584,7 +4815,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>35</v>
       </c>
@@ -4721,7 +4952,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>35</v>
       </c>
@@ -4858,19 +5089,19 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="23"/>
       <c r="B16" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="24"/>
       <c r="B17" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="25"/>
       <c r="B18" s="1" t="s">
         <v>128</v>

</xml_diff>